<commit_message>
fix: make C40(총납부액) independent of E39 chain to prevent #REF errors
Before: C40=IFERROR(E39,0) — deleting any cell in rows 35-39 breaks E39→C40
After:  C40 and all E35:E39 now compute directly from E31*(1-IFERROR(C35,0))*...

- Each E3x cell computes its balance directly from E31 × accumulated discount rates
- IFERROR(Cx,0) wraps each rate reference — deleted/errored cells treated as 0%
- D35:D39 still show per-step discount amounts (prev_balance - current_balance)
- C40, C41(=E39 equivalent), C42 all protected against #REF regardless of deletions

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/패키지 견적서(고정).xlsx
+++ b/패키지 견적서(고정).xlsx
@@ -3696,7 +3696,7 @@
         <v/>
       </c>
       <c r="E35" s="306">
-        <f>IFERROR(E31*(1-C35),E31)</f>
+        <f>IFERROR(E31*(1-IFERROR(C35,0)),IFERROR(E31,0))</f>
         <v/>
       </c>
       <c r="G35" s="17" t="inlineStr">
@@ -3721,7 +3721,7 @@
         <v/>
       </c>
       <c r="E36" s="306">
-        <f>IFERROR(E31*(1-C35)*(1-C36),E31)</f>
+        <f>IFERROR(E31*(1-IFERROR(C35,0))*(1-IFERROR(C36,0)),IFERROR(E31,0))</f>
         <v/>
       </c>
       <c r="G36" s="17" t="inlineStr">
@@ -3746,7 +3746,7 @@
         <v/>
       </c>
       <c r="E37" s="306">
-        <f>IFERROR(E31*(1-C35)*(1-C36)*(1-C37),E31)</f>
+        <f>IFERROR(E31*(1-IFERROR(C35,0))*(1-IFERROR(C36,0))*(1-IFERROR(C37,0)),IFERROR(E31,0))</f>
         <v/>
       </c>
       <c r="G37" s="17" t="inlineStr">
@@ -3771,7 +3771,7 @@
         <v/>
       </c>
       <c r="E38" s="306">
-        <f>IFERROR(E31*(1-C35)*(1-C36)*(1-C37)*(1-C38),E31)</f>
+        <f>IFERROR(E31*(1-IFERROR(C35,0))*(1-IFERROR(C36,0))*(1-IFERROR(C37,0))*(1-IFERROR(C38,0)),IFERROR(E31,0))</f>
         <v/>
       </c>
       <c r="G38" s="17" t="n"/>
@@ -3792,7 +3792,7 @@
         <v/>
       </c>
       <c r="E39" s="306">
-        <f>IFERROR(E31*(1-C35)*(1-C36)*(1-C37)*(1-C38)*(1-C39),E31)</f>
+        <f>IFERROR(E31*(1-IFERROR(C35,0))*(1-IFERROR(C36,0))*(1-IFERROR(C37,0))*(1-IFERROR(C38,0))*(1-IFERROR(C39,0)),IFERROR(E31,0))</f>
         <v/>
       </c>
       <c r="G39" s="17" t="n"/>
@@ -3808,7 +3808,7 @@
       </c>
       <c r="B40" s="307" t="n"/>
       <c r="C40" s="308">
-        <f>IFERROR(E39,0)</f>
+        <f>IFERROR(E31*(1-IFERROR(C35,0))*(1-IFERROR(C36,0))*(1-IFERROR(C37,0))*(1-IFERROR(C38,0))*(1-IFERROR(C39,0)),IFERROR(E31,0))</f>
         <v/>
       </c>
       <c r="D40" s="309" t="n"/>

</xml_diff>